<commit_message>
fix(data): correct mislabeled meat dishes in menu_items
19 dishes named after meat (pork spine soup, beef burger, goat curry, pork chop, steaks) were flagged contains_meat=0 / is_vegan=true. No-pork, vegan, and jay filters would have served them as safe. Corrected in menu_items.json and menu_items.xlsx.
</commit_message>
<xml_diff>
--- a/menu_items.xlsx
+++ b/menu_items.xlsx
@@ -2579,7 +2579,7 @@
         <v>0</v>
       </c>
       <c r="Q30" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R30" t="n">
         <v>0</v>
@@ -2650,13 +2650,13 @@
         <v>0</v>
       </c>
       <c r="Q31" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R31" t="n">
         <v>0</v>
       </c>
       <c r="S31" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T31" t="n">
         <v>0</v>
@@ -2863,13 +2863,13 @@
         <v>0</v>
       </c>
       <c r="Q34" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R34" t="n">
         <v>0</v>
       </c>
       <c r="S34" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T34" t="n">
         <v>0</v>
@@ -2934,7 +2934,7 @@
         <v>0</v>
       </c>
       <c r="Q35" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R35" t="n">
         <v>0</v>
@@ -33606,10 +33606,10 @@
         <v>0</v>
       </c>
       <c r="Q467" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R467" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S467" t="n">
         <v>0</v>
@@ -33677,10 +33677,10 @@
         <v>0</v>
       </c>
       <c r="Q468" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R468" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S468" t="n">
         <v>0</v>
@@ -33748,10 +33748,10 @@
         <v>0</v>
       </c>
       <c r="Q469" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R469" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S469" t="n">
         <v>0</v>
@@ -46954,7 +46954,7 @@
         <v>0</v>
       </c>
       <c r="Q655" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R655" t="n">
         <v>0</v>
@@ -46970,7 +46970,7 @@
       </c>
       <c r="V655" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>low</t>
         </is>
       </c>
       <c r="Y655" t="n">
@@ -47025,7 +47025,7 @@
         <v>0</v>
       </c>
       <c r="Q656" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R656" t="n">
         <v>0</v>
@@ -47041,7 +47041,7 @@
       </c>
       <c r="V656" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>low</t>
         </is>
       </c>
       <c r="Y656" t="n">
@@ -49581,7 +49581,7 @@
         <v>0</v>
       </c>
       <c r="Q692" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R692" t="n">
         <v>0</v>
@@ -55971,10 +55971,10 @@
         <v>0</v>
       </c>
       <c r="Q782" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R782" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S782" t="n">
         <v>0</v>
@@ -56042,7 +56042,7 @@
         <v>0</v>
       </c>
       <c r="Q783" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R783" t="n">
         <v>0</v>
@@ -61580,10 +61580,10 @@
         <v>0</v>
       </c>
       <c r="Q861" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R861" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S861" t="n">
         <v>0</v>
@@ -75283,13 +75283,13 @@
         <v>0</v>
       </c>
       <c r="Q1054" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R1054" t="n">
         <v>0</v>
       </c>
       <c r="S1054" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T1054" t="n">
         <v>0</v>
@@ -75354,13 +75354,13 @@
         <v>0</v>
       </c>
       <c r="Q1055" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R1055" t="n">
         <v>0</v>
       </c>
       <c r="S1055" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T1055" t="n">
         <v>0</v>
@@ -76845,7 +76845,7 @@
         <v>0</v>
       </c>
       <c r="Q1076" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R1076" t="n">
         <v>0</v>
@@ -76861,7 +76861,7 @@
       </c>
       <c r="V1076" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>low</t>
         </is>
       </c>
       <c r="Y1076" t="n">
@@ -84442,7 +84442,7 @@
         <v>0</v>
       </c>
       <c r="Q1183" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R1183" t="n">
         <v>0</v>
@@ -84513,7 +84513,7 @@
         <v>0</v>
       </c>
       <c r="Q1184" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R1184" t="n">
         <v>0</v>
@@ -84584,7 +84584,7 @@
         <v>0</v>
       </c>
       <c r="Q1185" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R1185" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
fix(data): label ingredients that dish names state outright
Adds flags the source data never set even though the dish name says so:
wheat on pasta, instant noodles, bread, pastries and pizza; soy on
teriyaki, sukiyaki and karaage; milk on latte, cappuccino, mocha and Thai
iced drinks; meat and pork on bacon dishes, nuggets and pork chop;
molluscs on takoyaki and scallop. Also clears flags the name rules out:
rice and glass noodles marked wheat, lamb and chicken marked beef,
chicken sausage marked pork.

159 rows in menu_items.json and menu_items.xlsx. Diet flags are re-derived
from the ingredient facts, not edited directly.

Limited to what the dish name states. Roughly 160 rows still under-labelled
where only the standard recipe implies an ingredient - egg in fried rice,
peanut in pad thai, squid in mixed seafood, pork in gyoza. Those need a
menu-by-menu pass, not a rule.
</commit_message>
<xml_diff>
--- a/menu_items.xlsx
+++ b/menu_items.xlsx
@@ -2567,7 +2567,7 @@
         <v>0</v>
       </c>
       <c r="M30" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N30" t="n">
         <v>0</v>
@@ -2638,7 +2638,7 @@
         <v>0</v>
       </c>
       <c r="M31" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N31" t="n">
         <v>0</v>
@@ -2709,7 +2709,7 @@
         <v>0</v>
       </c>
       <c r="M32" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N32" t="n">
         <v>0</v>
@@ -2780,7 +2780,7 @@
         <v>0</v>
       </c>
       <c r="M33" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N33" t="n">
         <v>0</v>
@@ -2851,7 +2851,7 @@
         <v>0</v>
       </c>
       <c r="M34" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N34" t="n">
         <v>0</v>
@@ -2922,7 +2922,7 @@
         <v>0</v>
       </c>
       <c r="M35" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N35" t="n">
         <v>0</v>
@@ -3076,7 +3076,7 @@
         <v>0</v>
       </c>
       <c r="Q37" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R37" t="n">
         <v>0</v>
@@ -3224,7 +3224,7 @@
         <v>0</v>
       </c>
       <c r="S39" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="T39" t="n">
         <v>0</v>
@@ -3295,7 +3295,7 @@
         <v>0</v>
       </c>
       <c r="S40" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="T40" t="n">
         <v>0</v>
@@ -3437,7 +3437,7 @@
         <v>0</v>
       </c>
       <c r="S42" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="T42" t="n">
         <v>0</v>
@@ -4082,7 +4082,7 @@
         <v>0</v>
       </c>
       <c r="U51" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V51" t="inlineStr">
         <is>
@@ -4129,7 +4129,7 @@
         <v>0</v>
       </c>
       <c r="M52" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N52" t="n">
         <v>0</v>
@@ -6898,7 +6898,7 @@
         <v>0</v>
       </c>
       <c r="M91" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N91" t="n">
         <v>0</v>
@@ -7466,7 +7466,7 @@
         <v>0</v>
       </c>
       <c r="M99" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N99" t="n">
         <v>0</v>
@@ -7478,7 +7478,7 @@
         <v>0</v>
       </c>
       <c r="Q99" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R99" t="n">
         <v>0</v>
@@ -8176,7 +8176,7 @@
         <v>0</v>
       </c>
       <c r="M109" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N109" t="n">
         <v>0</v>
@@ -8247,7 +8247,7 @@
         <v>0</v>
       </c>
       <c r="M110" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N110" t="n">
         <v>0</v>
@@ -8309,7 +8309,7 @@
         <v>1</v>
       </c>
       <c r="J111" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K111" t="n">
         <v>0</v>
@@ -8318,7 +8318,7 @@
         <v>0</v>
       </c>
       <c r="M111" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N111" t="n">
         <v>0</v>
@@ -8380,7 +8380,7 @@
         <v>1</v>
       </c>
       <c r="J112" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K112" t="n">
         <v>0</v>
@@ -8389,7 +8389,7 @@
         <v>0</v>
       </c>
       <c r="M112" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N112" t="n">
         <v>0</v>
@@ -8460,7 +8460,7 @@
         <v>0</v>
       </c>
       <c r="M113" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N113" t="n">
         <v>0</v>
@@ -8531,7 +8531,7 @@
         <v>0</v>
       </c>
       <c r="M114" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N114" t="n">
         <v>0</v>
@@ -8602,7 +8602,7 @@
         <v>0</v>
       </c>
       <c r="M115" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N115" t="n">
         <v>0</v>
@@ -8673,7 +8673,7 @@
         <v>0</v>
       </c>
       <c r="M116" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N116" t="n">
         <v>0</v>
@@ -8744,7 +8744,7 @@
         <v>0</v>
       </c>
       <c r="M117" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N117" t="n">
         <v>0</v>
@@ -9170,7 +9170,7 @@
         <v>0</v>
       </c>
       <c r="M123" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N123" t="n">
         <v>0</v>
@@ -9241,7 +9241,7 @@
         <v>0</v>
       </c>
       <c r="M124" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N124" t="n">
         <v>0</v>
@@ -9303,7 +9303,7 @@
         <v>1</v>
       </c>
       <c r="J125" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K125" t="n">
         <v>0</v>
@@ -9312,7 +9312,7 @@
         <v>0</v>
       </c>
       <c r="M125" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N125" t="n">
         <v>0</v>
@@ -9383,7 +9383,7 @@
         <v>0</v>
       </c>
       <c r="M126" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N126" t="n">
         <v>0</v>
@@ -9655,7 +9655,7 @@
         <v>0</v>
       </c>
       <c r="I130" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J130" t="n">
         <v>0</v>
@@ -9726,7 +9726,7 @@
         <v>0</v>
       </c>
       <c r="I131" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J131" t="n">
         <v>0</v>
@@ -10090,7 +10090,7 @@
         <v>0</v>
       </c>
       <c r="L136" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M136" t="n">
         <v>0</v>
@@ -12010,7 +12010,7 @@
         <v>0</v>
       </c>
       <c r="M163" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N163" t="n">
         <v>0</v>
@@ -12862,7 +12862,7 @@
         <v>0</v>
       </c>
       <c r="M175" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N175" t="n">
         <v>0</v>
@@ -14992,7 +14992,7 @@
         <v>0</v>
       </c>
       <c r="M205" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N205" t="n">
         <v>0</v>
@@ -15063,7 +15063,7 @@
         <v>0</v>
       </c>
       <c r="M206" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N206" t="n">
         <v>0</v>
@@ -15134,7 +15134,7 @@
         <v>0</v>
       </c>
       <c r="M207" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N207" t="n">
         <v>0</v>
@@ -15205,7 +15205,7 @@
         <v>0</v>
       </c>
       <c r="M208" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N208" t="n">
         <v>0</v>
@@ -15276,7 +15276,7 @@
         <v>0</v>
       </c>
       <c r="M209" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N209" t="n">
         <v>0</v>
@@ -15347,7 +15347,7 @@
         <v>0</v>
       </c>
       <c r="M210" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N210" t="n">
         <v>0</v>
@@ -15418,7 +15418,7 @@
         <v>0</v>
       </c>
       <c r="M211" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N211" t="n">
         <v>0</v>
@@ -15489,7 +15489,7 @@
         <v>0</v>
       </c>
       <c r="M212" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N212" t="n">
         <v>0</v>
@@ -15560,7 +15560,7 @@
         <v>0</v>
       </c>
       <c r="M213" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N213" t="n">
         <v>0</v>
@@ -15631,7 +15631,7 @@
         <v>0</v>
       </c>
       <c r="M214" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N214" t="n">
         <v>0</v>
@@ -15702,7 +15702,7 @@
         <v>0</v>
       </c>
       <c r="M215" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N215" t="n">
         <v>0</v>
@@ -15773,7 +15773,7 @@
         <v>0</v>
       </c>
       <c r="M216" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N216" t="n">
         <v>0</v>
@@ -15844,7 +15844,7 @@
         <v>0</v>
       </c>
       <c r="M217" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N217" t="n">
         <v>0</v>
@@ -15915,7 +15915,7 @@
         <v>0</v>
       </c>
       <c r="M218" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N218" t="n">
         <v>0</v>
@@ -15986,7 +15986,7 @@
         <v>0</v>
       </c>
       <c r="M219" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N219" t="n">
         <v>0</v>
@@ -16057,7 +16057,7 @@
         <v>0</v>
       </c>
       <c r="M220" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N220" t="n">
         <v>0</v>
@@ -16128,7 +16128,7 @@
         <v>0</v>
       </c>
       <c r="M221" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N221" t="n">
         <v>0</v>
@@ -18400,7 +18400,7 @@
         <v>0</v>
       </c>
       <c r="M253" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N253" t="n">
         <v>0</v>
@@ -18471,7 +18471,7 @@
         <v>0</v>
       </c>
       <c r="M254" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N254" t="n">
         <v>0</v>
@@ -18613,7 +18613,7 @@
         <v>0</v>
       </c>
       <c r="M256" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N256" t="n">
         <v>0</v>
@@ -20388,7 +20388,7 @@
         <v>0</v>
       </c>
       <c r="M281" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N281" t="n">
         <v>0</v>
@@ -20459,7 +20459,7 @@
         <v>0</v>
       </c>
       <c r="M282" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N282" t="n">
         <v>0</v>
@@ -21879,7 +21879,7 @@
         <v>0</v>
       </c>
       <c r="M302" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N302" t="n">
         <v>0</v>
@@ -21950,7 +21950,7 @@
         <v>0</v>
       </c>
       <c r="M303" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N303" t="n">
         <v>0</v>
@@ -22021,7 +22021,7 @@
         <v>0</v>
       </c>
       <c r="M304" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N304" t="n">
         <v>0</v>
@@ -22092,7 +22092,7 @@
         <v>0</v>
       </c>
       <c r="M305" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N305" t="n">
         <v>0</v>
@@ -22163,7 +22163,7 @@
         <v>0</v>
       </c>
       <c r="M306" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N306" t="n">
         <v>0</v>
@@ -22234,7 +22234,7 @@
         <v>0</v>
       </c>
       <c r="M307" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N307" t="n">
         <v>0</v>
@@ -24420,7 +24420,7 @@
         <v>0</v>
       </c>
       <c r="H338" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I338" t="n">
         <v>1</v>
@@ -29843,10 +29843,10 @@
         <v>0</v>
       </c>
       <c r="Q414" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R414" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S414" t="n">
         <v>0</v>
@@ -31535,7 +31535,7 @@
         <v>0</v>
       </c>
       <c r="M438" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N438" t="n">
         <v>1</v>
@@ -36727,7 +36727,7 @@
         <v>0</v>
       </c>
       <c r="P511" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q511" t="n">
         <v>0</v>
@@ -37437,7 +37437,7 @@
         <v>0</v>
       </c>
       <c r="P521" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q521" t="n">
         <v>0</v>
@@ -39688,7 +39688,7 @@
         <v>0</v>
       </c>
       <c r="I553" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J553" t="n">
         <v>0</v>
@@ -39830,7 +39830,7 @@
         <v>0</v>
       </c>
       <c r="I555" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J555" t="n">
         <v>0</v>
@@ -39984,7 +39984,7 @@
         <v>0</v>
       </c>
       <c r="M557" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N557" t="n">
         <v>0</v>
@@ -39996,7 +39996,7 @@
         <v>0</v>
       </c>
       <c r="Q557" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R557" t="n">
         <v>0</v>
@@ -40058,7 +40058,7 @@
         <v>0</v>
       </c>
       <c r="N558" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O558" t="n">
         <v>0</v>
@@ -40209,10 +40209,10 @@
         <v>0</v>
       </c>
       <c r="Q560" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R560" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S560" t="n">
         <v>0</v>
@@ -40351,10 +40351,10 @@
         <v>0</v>
       </c>
       <c r="Q562" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R562" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S562" t="n">
         <v>0</v>
@@ -40543,7 +40543,7 @@
         <v>0</v>
       </c>
       <c r="J565" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K565" t="n">
         <v>0</v>
@@ -40706,10 +40706,10 @@
         <v>0</v>
       </c>
       <c r="Q567" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R567" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S567" t="n">
         <v>0</v>
@@ -41265,7 +41265,7 @@
         <v>0</v>
       </c>
       <c r="N575" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O575" t="n">
         <v>0</v>
@@ -43321,7 +43321,7 @@
         <v>0</v>
       </c>
       <c r="M604" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N604" t="n">
         <v>0</v>
@@ -45028,7 +45028,7 @@
         <v>0</v>
       </c>
       <c r="N628" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O628" t="n">
         <v>0</v>
@@ -45522,7 +45522,7 @@
         <v>0</v>
       </c>
       <c r="M635" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N635" t="n">
         <v>1</v>
@@ -45593,7 +45593,7 @@
         <v>0</v>
       </c>
       <c r="M636" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N636" t="n">
         <v>0</v>
@@ -45877,7 +45877,7 @@
         <v>0</v>
       </c>
       <c r="M640" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N640" t="n">
         <v>0</v>
@@ -45889,7 +45889,7 @@
         <v>0</v>
       </c>
       <c r="Q640" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R640" t="n">
         <v>0</v>
@@ -46374,7 +46374,7 @@
         <v>0</v>
       </c>
       <c r="M647" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N647" t="n">
         <v>1</v>
@@ -46445,7 +46445,7 @@
         <v>0</v>
       </c>
       <c r="M648" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N648" t="n">
         <v>0</v>
@@ -46516,7 +46516,7 @@
         <v>0</v>
       </c>
       <c r="M649" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N649" t="n">
         <v>0</v>
@@ -46803,7 +46803,7 @@
         <v>0</v>
       </c>
       <c r="N653" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O653" t="n">
         <v>0</v>
@@ -47300,7 +47300,7 @@
         <v>0</v>
       </c>
       <c r="N660" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O660" t="n">
         <v>0</v>
@@ -47442,7 +47442,7 @@
         <v>0</v>
       </c>
       <c r="N662" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O662" t="n">
         <v>0</v>
@@ -47513,7 +47513,7 @@
         <v>0</v>
       </c>
       <c r="N663" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O663" t="n">
         <v>0</v>
@@ -47584,7 +47584,7 @@
         <v>0</v>
       </c>
       <c r="N664" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O664" t="n">
         <v>0</v>
@@ -49285,7 +49285,7 @@
         <v>0</v>
       </c>
       <c r="M688" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N688" t="n">
         <v>0</v>
@@ -49995,7 +49995,7 @@
         <v>0</v>
       </c>
       <c r="M698" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N698" t="n">
         <v>0</v>
@@ -50918,7 +50918,7 @@
         <v>0</v>
       </c>
       <c r="M711" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N711" t="n">
         <v>0</v>
@@ -51131,7 +51131,7 @@
         <v>0</v>
       </c>
       <c r="M714" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N714" t="n">
         <v>0</v>
@@ -51415,7 +51415,7 @@
         <v>0</v>
       </c>
       <c r="M718" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N718" t="n">
         <v>0</v>
@@ -51489,7 +51489,7 @@
         <v>1</v>
       </c>
       <c r="N719" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O719" t="n">
         <v>0</v>
@@ -51560,7 +51560,7 @@
         <v>0</v>
       </c>
       <c r="N720" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O720" t="n">
         <v>0</v>
@@ -51631,7 +51631,7 @@
         <v>0</v>
       </c>
       <c r="N721" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O721" t="n">
         <v>0</v>
@@ -52282,7 +52282,7 @@
         <v>1</v>
       </c>
       <c r="R730" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S730" t="n">
         <v>0</v>
@@ -52409,7 +52409,7 @@
         <v>0</v>
       </c>
       <c r="M732" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N732" t="n">
         <v>0</v>
@@ -52551,7 +52551,7 @@
         <v>0</v>
       </c>
       <c r="M734" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N734" t="n">
         <v>0</v>
@@ -52622,7 +52622,7 @@
         <v>0</v>
       </c>
       <c r="M735" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N735" t="n">
         <v>0</v>
@@ -52693,7 +52693,7 @@
         <v>0</v>
       </c>
       <c r="M736" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N736" t="n">
         <v>0</v>
@@ -53110,7 +53110,7 @@
         <v>0</v>
       </c>
       <c r="J742" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K742" t="n">
         <v>0</v>
@@ -53474,7 +53474,7 @@
         <v>0</v>
       </c>
       <c r="M747" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N747" t="n">
         <v>0</v>
@@ -53545,7 +53545,7 @@
         <v>0</v>
       </c>
       <c r="M748" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N748" t="n">
         <v>0</v>
@@ -53616,7 +53616,7 @@
         <v>0</v>
       </c>
       <c r="M749" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N749" t="n">
         <v>0</v>
@@ -53687,7 +53687,7 @@
         <v>0</v>
       </c>
       <c r="M750" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N750" t="n">
         <v>0</v>
@@ -53758,7 +53758,7 @@
         <v>1</v>
       </c>
       <c r="M751" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N751" t="n">
         <v>0</v>
@@ -53971,7 +53971,7 @@
         <v>0</v>
       </c>
       <c r="M754" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N754" t="n">
         <v>0</v>
@@ -54042,7 +54042,7 @@
         <v>0</v>
       </c>
       <c r="M755" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N755" t="n">
         <v>0</v>
@@ -54480,10 +54480,10 @@
         <v>0</v>
       </c>
       <c r="Q761" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R761" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S761" t="n">
         <v>0</v>
@@ -54752,7 +54752,7 @@
         <v>0</v>
       </c>
       <c r="M765" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N765" t="n">
         <v>0</v>
@@ -54823,7 +54823,7 @@
         <v>0</v>
       </c>
       <c r="M766" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N766" t="n">
         <v>0</v>
@@ -54894,7 +54894,7 @@
         <v>0</v>
       </c>
       <c r="M767" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N767" t="n">
         <v>0</v>
@@ -54965,7 +54965,7 @@
         <v>0</v>
       </c>
       <c r="M768" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N768" t="n">
         <v>0</v>
@@ -55394,7 +55394,7 @@
         <v>0</v>
       </c>
       <c r="N774" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O774" t="n">
         <v>0</v>
@@ -56104,7 +56104,7 @@
         <v>0</v>
       </c>
       <c r="N784" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O784" t="n">
         <v>0</v>
@@ -56527,7 +56527,7 @@
         <v>0</v>
       </c>
       <c r="M790" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N790" t="n">
         <v>0</v>
@@ -57379,7 +57379,7 @@
         <v>0</v>
       </c>
       <c r="M802" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N802" t="n">
         <v>0</v>
@@ -57521,7 +57521,7 @@
         <v>0</v>
       </c>
       <c r="M804" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N804" t="n">
         <v>0</v>
@@ -57947,7 +57947,7 @@
         <v>0</v>
       </c>
       <c r="M810" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N810" t="n">
         <v>0</v>
@@ -59237,10 +59237,10 @@
         <v>0</v>
       </c>
       <c r="Q828" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R828" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S828" t="n">
         <v>0</v>
@@ -59592,13 +59592,13 @@
         <v>0</v>
       </c>
       <c r="Q833" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R833" t="n">
         <v>0</v>
       </c>
       <c r="S833" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T833" t="n">
         <v>0</v>
@@ -60018,7 +60018,7 @@
         <v>0</v>
       </c>
       <c r="Q839" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R839" t="n">
         <v>0</v>
@@ -62420,7 +62420,7 @@
         <v>0</v>
       </c>
       <c r="M873" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N873" t="n">
         <v>0</v>
@@ -63636,7 +63636,7 @@
         <v>0</v>
       </c>
       <c r="P890" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q890" t="n">
         <v>0</v>
@@ -64411,7 +64411,7 @@
         <v>1</v>
       </c>
       <c r="N901" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O901" t="n">
         <v>0</v>
@@ -65911,10 +65911,10 @@
         <v>0</v>
       </c>
       <c r="Q922" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R922" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S922" t="n">
         <v>0</v>
@@ -65927,7 +65927,7 @@
       </c>
       <c r="V922" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>high</t>
         </is>
       </c>
       <c r="Y922" t="n">
@@ -66254,7 +66254,7 @@
         <v>0</v>
       </c>
       <c r="M927" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N927" t="n">
         <v>0</v>
@@ -66325,7 +66325,7 @@
         <v>0</v>
       </c>
       <c r="M928" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N928" t="n">
         <v>0</v>
@@ -66538,7 +66538,7 @@
         <v>0</v>
       </c>
       <c r="M931" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N931" t="n">
         <v>0</v>
@@ -66683,7 +66683,7 @@
         <v>0</v>
       </c>
       <c r="N933" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O933" t="n">
         <v>0</v>
@@ -66964,7 +66964,7 @@
         <v>0</v>
       </c>
       <c r="M937" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N937" t="n">
         <v>0</v>
@@ -68017,7 +68017,7 @@
         <v>0</v>
       </c>
       <c r="I952" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J952" t="n">
         <v>0</v>
@@ -68088,7 +68088,7 @@
         <v>0</v>
       </c>
       <c r="I953" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J953" t="n">
         <v>0</v>
@@ -68159,7 +68159,7 @@
         <v>0</v>
       </c>
       <c r="I954" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J954" t="n">
         <v>0</v>
@@ -68301,7 +68301,7 @@
         <v>0</v>
       </c>
       <c r="I956" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J956" t="n">
         <v>0</v>
@@ -68384,7 +68384,7 @@
         <v>0</v>
       </c>
       <c r="M957" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N957" t="n">
         <v>0</v>
@@ -68526,7 +68526,7 @@
         <v>0</v>
       </c>
       <c r="M959" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N959" t="n">
         <v>0</v>
@@ -68810,7 +68810,7 @@
         <v>0</v>
       </c>
       <c r="M963" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N963" t="n">
         <v>0</v>
@@ -70230,7 +70230,7 @@
         <v>0</v>
       </c>
       <c r="M983" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N983" t="n">
         <v>0</v>
@@ -70455,10 +70455,10 @@
         <v>0</v>
       </c>
       <c r="Q986" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R986" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S986" t="n">
         <v>0</v>
@@ -71721,7 +71721,7 @@
         <v>0</v>
       </c>
       <c r="M1004" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N1004" t="n">
         <v>0</v>
@@ -75141,13 +75141,13 @@
         <v>0</v>
       </c>
       <c r="Q1052" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R1052" t="n">
         <v>0</v>
       </c>
       <c r="S1052" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T1052" t="n">
         <v>0</v>
@@ -75697,7 +75697,7 @@
         <v>0</v>
       </c>
       <c r="M1060" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N1060" t="n">
         <v>0</v>
@@ -76987,10 +76987,10 @@
         <v>0</v>
       </c>
       <c r="Q1078" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R1078" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S1078" t="n">
         <v>0</v>
@@ -77003,7 +77003,7 @@
       </c>
       <c r="V1078" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>high</t>
         </is>
       </c>
       <c r="Y1078" t="n">
@@ -77070,7 +77070,7 @@
         <v>0</v>
       </c>
       <c r="U1079" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V1079" t="inlineStr">
         <is>
@@ -81155,7 +81155,7 @@
         <v>1</v>
       </c>
       <c r="J1137" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K1137" t="n">
         <v>0</v>
@@ -82880,13 +82880,13 @@
         <v>0</v>
       </c>
       <c r="Q1161" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R1161" t="n">
         <v>0</v>
       </c>
       <c r="S1161" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="T1161" t="n">
         <v>0</v>
@@ -83152,7 +83152,7 @@
         <v>0</v>
       </c>
       <c r="M1165" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N1165" t="n">
         <v>0</v>
@@ -83161,7 +83161,7 @@
         <v>0</v>
       </c>
       <c r="P1165" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q1165" t="n">
         <v>0</v>
@@ -84300,7 +84300,7 @@
         <v>0</v>
       </c>
       <c r="Q1181" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R1181" t="n">
         <v>0</v>
@@ -84371,7 +84371,7 @@
         <v>0</v>
       </c>
       <c r="Q1182" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R1182" t="n">
         <v>0</v>
@@ -84643,7 +84643,7 @@
         <v>0</v>
       </c>
       <c r="M1186" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N1186" t="n">
         <v>0</v>
@@ -84785,7 +84785,7 @@
         <v>0</v>
       </c>
       <c r="M1188" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N1188" t="n">
         <v>0</v>
@@ -84856,7 +84856,7 @@
         <v>0</v>
       </c>
       <c r="M1189" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N1189" t="n">
         <v>0</v>
@@ -84927,7 +84927,7 @@
         <v>0</v>
       </c>
       <c r="M1190" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N1190" t="n">
         <v>0</v>
@@ -85770,7 +85770,7 @@
         <v>1</v>
       </c>
       <c r="J1202" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K1202" t="n">
         <v>0</v>
@@ -86560,7 +86560,7 @@
         <v>0</v>
       </c>
       <c r="M1213" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N1213" t="n">
         <v>0</v>
@@ -87285,7 +87285,7 @@
         <v>1</v>
       </c>
       <c r="R1223" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S1223" t="n">
         <v>0</v>
@@ -87708,10 +87708,10 @@
         <v>0</v>
       </c>
       <c r="Q1229" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R1229" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S1229" t="n">
         <v>0</v>
@@ -88196,7 +88196,7 @@
         <v>0</v>
       </c>
       <c r="N1236" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O1236" t="n">
         <v>0</v>
@@ -88974,7 +88974,7 @@
         <v>0</v>
       </c>
       <c r="M1247" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N1247" t="n">
         <v>0</v>
@@ -89258,7 +89258,7 @@
         <v>0</v>
       </c>
       <c r="M1251" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N1251" t="n">
         <v>0</v>

</xml_diff>